<commit_message>
fix: keep control sheet failures row-local
</commit_message>
<xml_diff>
--- a/tests/fixtures/control-sheet-cases.xlsx
+++ b/tests/fixtures/control-sheet-cases.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Controle" sheetId="1" r:id="rId1"/>
+    <sheet name="Resumo" sheetId="1" r:id="rId1"/>
+    <sheet name="LV e Site" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -18,12 +19,15 @@
   <borders count="1">
     <border/>
   </borders>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <cellStyleXfs count="1">
     <xf/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0"/>
-    <xf numFmtId="14" applyNumberFormat="1"/>
+    <xf numFmtId="164" applyNumberFormat="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -34,6 +38,20 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Resumo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t> Titulo </t>
         </is>
       </c>
@@ -391,46 +409,138 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>011547/2026</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>72-2026</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Implantacao de Loja Virtual</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>18573230000105</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>CASA NOSSA</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Christian Albuquerque Alonso</t>
         </is>
       </c>
-      <c r="G9" s="1">
+      <c r="G10" s="1">
         <v>46133</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>https://out-of-scope.example/</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>012000/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>80-2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Insercao digital - Desenvolvimento de WebSite</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CNPJ INVALIDO</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Bruno Henrique Santana Leal</t>
+        </is>
+      </c>
+      <c r="G11" s="1">
+        <v>46150</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://invalid-cnpj.example/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>012001/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>81-2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Insercao digital - Desenvolvimento de WebSite</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>52999999000199</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>KICK OFF INVALIDO</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Bruno Henrique Santana Leal</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>amanha</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://invalid-kickoff.example/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
feat: generate reports from control rows (#8)
</commit_message>
<xml_diff>
--- a/tests/fixtures/control-sheet-cases.xlsx
+++ b/tests/fixtures/control-sheet-cases.xlsx
@@ -546,6 +546,51 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>012099/2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>40-2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Insercao digital - Desenvolvimento de WebSite</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>11222333000181</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>EMPRESA GEMEA LTDA</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Christian Albuquerque Alonso</t>
+        </is>
+      </c>
+      <c r="G14" s="1">
+        <v>46185</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://gemea.example/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cover Loja Virtual rows from the committed fixture, not the real sheet
tests/test_loja_virtual.py read `referencias/Planilha para controle de
relatórios.xlsx`, which is gitignored, so four of the five Loja tests
errored in CI and the Tema routing was only ever proven locally.

The fixture generator had also drifted from the committed workbook: it
moved `Implantacao de Loja Virtual` out of the out-of-scope slot without
putting a Loja row back, leaving no row that exercises `UnsupportedRow`.

Give the fixture its own Loja Virtual rows — one selectable, one stopped
on an invalid CNPJ — plus a genuinely unsupported Tema, and match Temas
through the routing contract so a row keeps the sheet's own spelling.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/control-sheet-cases.xlsx
+++ b/tests/fixtures/control-sheet-cases.xlsx
@@ -445,7 +445,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://out-of-scope.example/</t>
+          <t>https://casanossa.example/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -631,6 +631,96 @@
         </is>
       </c>
       <c r="I16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>012140/2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>46-2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Implantacao de Loja Virtual</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LOJA CNPJ INVALIDO</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Christian Albuquerque Alonso</t>
+        </is>
+      </c>
+      <c r="G17" s="1">
+        <v>46164</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://loja-invalida.example/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>012160/2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>47-2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Servico sem Master aprovado</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>30129441000160</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SERVICO NAO CONTRATADO</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Bruno Henrique Santana Leal</t>
+        </is>
+      </c>
+      <c r="G19" s="1">
+        <v>46168</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://out-of-scope.example/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>